<commit_message>
Add international TDK management workflow
</commit_message>
<xml_diff>
--- a/办公软件/111/templates/TDK配置模板.xlsx
+++ b/办公软件/111/templates/TDK配置模板.xlsx
@@ -7,8 +7,8 @@
     <sheet name="填写说明" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'TDK配置'!A1:L2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'填写说明'!A1:C13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'TDK配置'!A1:D1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'填写说明'!A1:C5</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -402,113 +402,43 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:D1"/>
   <cols>
-    <col min="1" max="1" width="14.83203125" customWidth="1"/>
-    <col min="2" max="2" width="28.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="18.83203125" customWidth="1"/>
-    <col min="6" max="6" width="48.83203125" customWidth="1"/>
-    <col min="7" max="7" width="22.83203125" customWidth="1"/>
-    <col min="8" max="8" width="42.83203125" customWidth="1"/>
-    <col min="9" max="9" width="60.83203125" customWidth="1"/>
-    <col min="10" max="10" width="34.83203125" customWidth="1"/>
-    <col min="11" max="11" width="12.83203125" customWidth="1"/>
-    <col min="12" max="12" width="34.83203125" customWidth="1"/>
+    <col min="1" max="1" width="48.83203125" customWidth="1"/>
+    <col min="2" max="2" width="52.83203125" customWidth="1"/>
+    <col min="3" max="3" width="42.83203125" customWidth="1"/>
+    <col min="4" max="4" width="72.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Record ID</v>
+        <v>Url Path</v>
       </c>
       <c r="B1" t="str">
-        <v>Site URL</v>
+        <v>Title</v>
       </c>
       <c r="C1" t="str">
-        <v>Site Code</v>
+        <v>Keyword</v>
       </c>
       <c r="D1" t="str">
-        <v>Language</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Page Type</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Page URL</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Product</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Title</v>
-      </c>
-      <c r="I1" t="str">
-        <v>Description</v>
-      </c>
-      <c r="J1" t="str">
-        <v>Keywords</v>
-      </c>
-      <c r="K1" t="str">
-        <v>Action</v>
-      </c>
-      <c r="L1" t="str">
-        <v>Notes</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>TDK-0001</v>
-      </c>
-      <c r="B2" t="str">
-        <v>https://www.ezviz.com/id</v>
-      </c>
-      <c r="C2" t="str">
-        <v>id</v>
-      </c>
-      <c r="D2" t="str">
-        <v>id-ID</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Product Detail</v>
-      </c>
-      <c r="F2" t="str">
-        <v>https://www.ezviz.com/id/product/example/00000</v>
-      </c>
-      <c r="G2" t="str">
-        <v>Example Product</v>
-      </c>
-      <c r="H2" t="str">
-        <v>Example Product | EZVIZ</v>
-      </c>
-      <c r="I2" t="str">
-        <v>Describe the page in the site language.</v>
-      </c>
-      <c r="J2" t="str">
-        <v>example product, ezviz</v>
-      </c>
-      <c r="K2" t="str">
-        <v>update</v>
-      </c>
-      <c r="L2" t="str">
-        <v>示例行，正式填写时请删除</v>
+        <v>Discription</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L2"/>
+  <autoFilter ref="A1:D1"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C5"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="72.83203125" customWidth="1"/>
+    <col min="3" max="3" width="88.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -524,140 +454,52 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Record ID</v>
+        <v>Url Path</v>
       </c>
       <c r="B2" t="str">
         <v>是</v>
       </c>
       <c r="C2" t="str">
-        <v>每行唯一且长期稳定，例如 TDK-0001</v>
+        <v>国际站相对路径，以 / 开头，例如 /inter/product/example/00000；不要填写域名</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Site URL</v>
+        <v>Title</v>
       </c>
       <c r="B3" t="str">
         <v>是</v>
       </c>
       <c r="C3" t="str">
-        <v>站点首页 URL，用于识别目标站点</v>
+        <v>对应后台 Title 字段；建议清晰、唯一，并包含核心主题</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Site Code</v>
+        <v>Keyword</v>
       </c>
       <c r="B4" t="str">
-        <v>否</v>
+        <v>是</v>
       </c>
       <c r="C4" t="str">
-        <v>站点代码；未知时可留空，后续优先按 Site URL 识别</v>
+        <v>对应后台 Keyword 字段；多个关键词建议使用英文逗号分隔</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Language</v>
+        <v>Discription</v>
       </c>
       <c r="B5" t="str">
         <v>是</v>
       </c>
       <c r="C5" t="str">
-        <v>页面语言代码，例如 en-US、id-ID、tr-TR</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Page Type</v>
-      </c>
-      <c r="B6" t="str">
-        <v>是</v>
-      </c>
-      <c r="C6" t="str">
-        <v>建议：Home、Category、Product Detail、Support、Campaign、Other</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Page URL</v>
-      </c>
-      <c r="B7" t="str">
-        <v>是</v>
-      </c>
-      <c r="C7" t="str">
-        <v>需要配置 TDK 的完整页面 URL</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Product</v>
-      </c>
-      <c r="B8" t="str">
-        <v>否</v>
-      </c>
-      <c r="C8" t="str">
-        <v>产品页填写产品名，其他页面可留空</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Title</v>
-      </c>
-      <c r="B9" t="str">
-        <v>是</v>
-      </c>
-      <c r="C9" t="str">
-        <v>页面 Title；建议清晰、唯一，并包含核心主题</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>Description</v>
-      </c>
-      <c r="B10" t="str">
-        <v>是</v>
-      </c>
-      <c r="C10" t="str">
-        <v>页面描述；使用对应站点语言，避免与其他页面重复</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>Keywords</v>
-      </c>
-      <c r="B11" t="str">
-        <v>否</v>
-      </c>
-      <c r="C11" t="str">
-        <v>关键词用英文逗号分隔；后台不需要时可留空</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>Action</v>
-      </c>
-      <c r="B12" t="str">
-        <v>否</v>
-      </c>
-      <c r="C12" t="str">
-        <v>create、update 或 skip；默认按 update 处理</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>Notes</v>
-      </c>
-      <c r="B13" t="str">
-        <v>否</v>
-      </c>
-      <c r="C13" t="str">
-        <v>特殊要求、人工确认事项或错误说明</v>
+        <v>对应后台 Discription 字段（沿用后台拼写）；填写页面描述</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C13"/>
+  <autoFilter ref="A1:C5"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>